<commit_message>
s8 demo: reviewer polish - size filler households to their units, tighten E3/E6/E10 rule wording
</commit_message>
<xml_diff>
--- a/backend/benchmark_data/s8_demo/rent_roll/oak_hollow_rent_roll_40unit.xlsx
+++ b/backend/benchmark_data/s8_demo/rent_roll/oak_hollow_rent_roll_40unit.xlsx
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>44774</v>
@@ -631,10 +631,10 @@
         <v>110</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>915</v>
+        <v>927</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>0</v>
@@ -731,7 +731,7 @@
         <v>4</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>43862</v>
+        <v>45047</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -739,10 +739,10 @@
         </is>
       </c>
       <c r="I9" s="3" t="n">
-        <v>46054</v>
+        <v>46143</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="K9" s="4" t="n">
         <v>1240</v>
@@ -751,10 +751,10 @@
         <v>110</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>498</v>
+        <v>698</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>742</v>
+        <v>542</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>0</v>
@@ -788,10 +788,10 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>44228</v>
+        <v>42583</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -799,10 +799,10 @@
         </is>
       </c>
       <c r="I10" s="3" t="n">
-        <v>46054</v>
+        <v>46235</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>46419</v>
+        <v>46600</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>1240</v>
@@ -811,10 +811,10 @@
         <v>110</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>615</v>
+        <v>287</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>625</v>
+        <v>953</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>0</v>
@@ -908,10 +908,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>41974</v>
+        <v>44378</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="I12" s="3" t="n">
-        <v>45992</v>
+        <v>46204</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>46357</v>
+        <v>46569</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>1240</v>
@@ -931,10 +931,10 @@
         <v>110</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>259</v>
+        <v>193</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>981</v>
+        <v>1047</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>0</v>
@@ -971,7 +971,7 @@
         <v>2</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>42675</v>
+        <v>44531</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -979,10 +979,10 @@
         </is>
       </c>
       <c r="I13" s="3" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="K13" s="4" t="n">
         <v>1050</v>
@@ -991,10 +991,10 @@
         <v>85</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>620</v>
+        <v>145</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>430</v>
+        <v>905</v>
       </c>
       <c r="O13" s="4" t="n">
         <v>0</v>
@@ -1088,10 +1088,10 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>42491</v>
+        <v>43282</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1099,10 +1099,10 @@
         </is>
       </c>
       <c r="I15" s="3" t="n">
-        <v>46143</v>
+        <v>46204</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>46508</v>
+        <v>46569</v>
       </c>
       <c r="K15" s="4" t="n">
         <v>1240</v>
@@ -1111,10 +1111,10 @@
         <v>110</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>835</v>
+        <v>803</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>405</v>
+        <v>437</v>
       </c>
       <c r="O15" s="4" t="n">
         <v>0</v>
@@ -1148,10 +1148,10 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>45352</v>
+        <v>44593</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1159,10 +1159,10 @@
         </is>
       </c>
       <c r="I16" s="3" t="n">
-        <v>46082</v>
+        <v>46054</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="K16" s="4" t="n">
         <v>1050</v>
@@ -1171,10 +1171,10 @@
         <v>85</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>715</v>
+        <v>781</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>335</v>
+        <v>269</v>
       </c>
       <c r="O16" s="4" t="n">
         <v>0</v>
@@ -1208,10 +1208,10 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>44593</v>
+        <v>43435</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1219,10 +1219,10 @@
         </is>
       </c>
       <c r="I17" s="3" t="n">
-        <v>46054</v>
+        <v>45992</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>46419</v>
+        <v>46357</v>
       </c>
       <c r="K17" s="4" t="n">
         <v>1240</v>
@@ -1231,10 +1231,10 @@
         <v>110</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>756</v>
+        <v>674</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>484</v>
+        <v>566</v>
       </c>
       <c r="O17" s="4" t="n">
         <v>0</v>
@@ -1268,10 +1268,10 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>43435</v>
+        <v>42887</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1279,10 +1279,10 @@
         </is>
       </c>
       <c r="I18" s="3" t="n">
-        <v>45992</v>
+        <v>46174</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>46357</v>
+        <v>46539</v>
       </c>
       <c r="K18" s="4" t="n">
         <v>1240</v>
@@ -1291,10 +1291,10 @@
         <v>110</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>438</v>
+        <v>212</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>802</v>
+        <v>1028</v>
       </c>
       <c r="O18" s="4" t="n">
         <v>0</v>
@@ -1388,10 +1388,10 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>42887</v>
+        <v>44743</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1399,10 +1399,10 @@
         </is>
       </c>
       <c r="I20" s="3" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>46539</v>
+        <v>46569</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>1240</v>
@@ -1411,10 +1411,10 @@
         <v>110</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>224</v>
+        <v>765</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>1016</v>
+        <v>475</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>0</v>
@@ -1451,7 +1451,7 @@
         <v>2</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>41883</v>
+        <v>43160</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1459,10 +1459,10 @@
         </is>
       </c>
       <c r="I21" s="3" t="n">
-        <v>46266</v>
+        <v>46082</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>46631</v>
+        <v>46447</v>
       </c>
       <c r="K21" s="4" t="n">
         <v>1050</v>
@@ -1471,10 +1471,10 @@
         <v>85</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>313</v>
+        <v>210</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>737</v>
+        <v>840</v>
       </c>
       <c r="O21" s="4" t="n">
         <v>0</v>
@@ -1628,10 +1628,10 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>44896</v>
+        <v>41671</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1639,10 +1639,10 @@
         </is>
       </c>
       <c r="I24" s="3" t="n">
-        <v>45992</v>
+        <v>46054</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>46357</v>
+        <v>46419</v>
       </c>
       <c r="K24" s="4" t="n">
         <v>1480</v>
@@ -1651,10 +1651,10 @@
         <v>135</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>617</v>
+        <v>493</v>
       </c>
       <c r="N24" s="4" t="n">
-        <v>863</v>
+        <v>987</v>
       </c>
       <c r="O24" s="4" t="n">
         <v>0</v>
@@ -1688,10 +1688,10 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>44682</v>
+        <v>44378</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1699,10 +1699,10 @@
         </is>
       </c>
       <c r="I25" s="3" t="n">
-        <v>46143</v>
+        <v>46204</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>46508</v>
+        <v>46569</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>1240</v>
@@ -1711,10 +1711,10 @@
         <v>110</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>386</v>
+        <v>784</v>
       </c>
       <c r="N25" s="4" t="n">
-        <v>854</v>
+        <v>456</v>
       </c>
       <c r="O25" s="4" t="n">
         <v>0</v>
@@ -1748,10 +1748,10 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>45536</v>
+        <v>44013</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1759,10 +1759,10 @@
         </is>
       </c>
       <c r="I26" s="3" t="n">
-        <v>46266</v>
+        <v>46204</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>46631</v>
+        <v>46569</v>
       </c>
       <c r="K26" s="4" t="n">
         <v>1050</v>
@@ -1771,10 +1771,10 @@
         <v>85</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>157</v>
+        <v>787</v>
       </c>
       <c r="N26" s="4" t="n">
-        <v>893</v>
+        <v>263</v>
       </c>
       <c r="O26" s="4" t="n">
         <v>0</v>
@@ -1868,10 +1868,10 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>43344</v>
+        <v>43497</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1879,10 +1879,10 @@
         </is>
       </c>
       <c r="I28" s="3" t="n">
-        <v>46266</v>
+        <v>46054</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>46631</v>
+        <v>46419</v>
       </c>
       <c r="K28" s="4" t="n">
         <v>1240</v>
@@ -1891,10 +1891,10 @@
         <v>110</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>590</v>
+        <v>372</v>
       </c>
       <c r="N28" s="4" t="n">
-        <v>650</v>
+        <v>868</v>
       </c>
       <c r="O28" s="4" t="n">
         <v>0</v>
@@ -1931,7 +1931,7 @@
         <v>3</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>44256</v>
+        <v>43525</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -1951,10 +1951,10 @@
         <v>110</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>511</v>
+        <v>417</v>
       </c>
       <c r="N29" s="4" t="n">
-        <v>729</v>
+        <v>823</v>
       </c>
       <c r="O29" s="4" t="n">
         <v>0</v>
@@ -2048,10 +2048,10 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>41730</v>
+        <v>44652</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -2071,10 +2071,10 @@
         <v>85</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>492</v>
+        <v>310</v>
       </c>
       <c r="N31" s="4" t="n">
-        <v>558</v>
+        <v>740</v>
       </c>
       <c r="O31" s="4" t="n">
         <v>0</v>
@@ -2111,7 +2111,7 @@
         <v>2</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>44562</v>
+        <v>42036</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -2119,10 +2119,10 @@
         </is>
       </c>
       <c r="I32" s="3" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="K32" s="4" t="n">
         <v>1240</v>
@@ -2131,10 +2131,10 @@
         <v>110</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>454</v>
+        <v>746</v>
       </c>
       <c r="N32" s="4" t="n">
-        <v>786</v>
+        <v>494</v>
       </c>
       <c r="O32" s="4" t="n">
         <v>0</v>
@@ -2228,10 +2228,10 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>45139</v>
+        <v>43405</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -2239,10 +2239,10 @@
         </is>
       </c>
       <c r="I34" s="3" t="n">
-        <v>46235</v>
+        <v>45962</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>46600</v>
+        <v>46327</v>
       </c>
       <c r="K34" s="4" t="n">
         <v>1480</v>
@@ -2251,10 +2251,10 @@
         <v>135</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>611</v>
+        <v>159</v>
       </c>
       <c r="N34" s="4" t="n">
-        <v>869</v>
+        <v>1321</v>
       </c>
       <c r="O34" s="4" t="n">
         <v>0</v>
@@ -2348,10 +2348,10 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>44166</v>
+        <v>45444</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2359,10 +2359,10 @@
         </is>
       </c>
       <c r="I36" s="3" t="n">
-        <v>45992</v>
+        <v>46174</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>46357</v>
+        <v>46539</v>
       </c>
       <c r="K36" s="4" t="n">
         <v>1050</v>
@@ -2371,10 +2371,10 @@
         <v>85</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>845</v>
+        <v>467</v>
       </c>
       <c r="N36" s="4" t="n">
-        <v>205</v>
+        <v>583</v>
       </c>
       <c r="O36" s="4" t="n">
         <v>0</v>
@@ -2408,10 +2408,10 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>42064</v>
+        <v>42826</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2419,10 +2419,10 @@
         </is>
       </c>
       <c r="I37" s="3" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="K37" s="4" t="n">
         <v>1240</v>
@@ -2431,10 +2431,10 @@
         <v>110</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>548</v>
+        <v>370</v>
       </c>
       <c r="N37" s="4" t="n">
-        <v>692</v>
+        <v>870</v>
       </c>
       <c r="O37" s="4" t="n">
         <v>0</v>
@@ -2516,10 +2516,10 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>44805</v>
+        <v>41791</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -2527,10 +2527,10 @@
         </is>
       </c>
       <c r="I39" s="3" t="n">
-        <v>46266</v>
+        <v>46174</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>46631</v>
+        <v>46539</v>
       </c>
       <c r="K39" s="4" t="n">
         <v>1240</v>
@@ -2539,10 +2539,10 @@
         <v>110</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>108</v>
+        <v>316</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>1132</v>
+        <v>924</v>
       </c>
       <c r="O39" s="4" t="n">
         <v>0</v>
@@ -2576,10 +2576,10 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>42826</v>
+        <v>42948</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -2587,10 +2587,10 @@
         </is>
       </c>
       <c r="I40" s="3" t="n">
-        <v>46113</v>
+        <v>46235</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>46478</v>
+        <v>46600</v>
       </c>
       <c r="K40" s="4" t="n">
         <v>1240</v>
@@ -2599,10 +2599,10 @@
         <v>110</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>370</v>
+        <v>449</v>
       </c>
       <c r="N40" s="4" t="n">
-        <v>870</v>
+        <v>791</v>
       </c>
       <c r="O40" s="4" t="n">
         <v>0</v>
@@ -2636,10 +2636,10 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>41791</v>
+        <v>44013</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -2647,10 +2647,10 @@
         </is>
       </c>
       <c r="I41" s="3" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>46539</v>
+        <v>46569</v>
       </c>
       <c r="K41" s="4" t="n">
         <v>1050</v>
@@ -2659,10 +2659,10 @@
         <v>85</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>365</v>
+        <v>244</v>
       </c>
       <c r="N41" s="4" t="n">
-        <v>685</v>
+        <v>806</v>
       </c>
       <c r="O41" s="4" t="n">
         <v>0</v>
@@ -2696,10 +2696,10 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>42948</v>
+        <v>43040</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -2707,10 +2707,10 @@
         </is>
       </c>
       <c r="I42" s="3" t="n">
-        <v>46235</v>
+        <v>45962</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>46600</v>
+        <v>46327</v>
       </c>
       <c r="K42" s="4" t="n">
         <v>1240</v>
@@ -2719,10 +2719,10 @@
         <v>110</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>449</v>
+        <v>293</v>
       </c>
       <c r="N42" s="4" t="n">
-        <v>791</v>
+        <v>947</v>
       </c>
       <c r="O42" s="4" t="n">
         <v>0</v>
@@ -2759,7 +2759,7 @@
         <v>1</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>44013</v>
+        <v>43983</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -2767,10 +2767,10 @@
         </is>
       </c>
       <c r="I43" s="3" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>46569</v>
+        <v>46539</v>
       </c>
       <c r="K43" s="4" t="n">
         <v>1050</v>
@@ -2779,10 +2779,10 @@
         <v>85</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>244</v>
+        <v>582</v>
       </c>
       <c r="N43" s="4" t="n">
-        <v>806</v>
+        <v>468</v>
       </c>
       <c r="O43" s="4" t="n">
         <v>0</v>
@@ -2816,10 +2816,10 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>43040</v>
+        <v>42767</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -2827,10 +2827,10 @@
         </is>
       </c>
       <c r="I44" s="3" t="n">
-        <v>45962</v>
+        <v>46054</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>46327</v>
+        <v>46419</v>
       </c>
       <c r="K44" s="4" t="n">
         <v>1480</v>
@@ -2839,10 +2839,10 @@
         <v>135</v>
       </c>
       <c r="M44" s="4" t="n">
-        <v>280</v>
+        <v>66</v>
       </c>
       <c r="N44" s="4" t="n">
-        <v>1200</v>
+        <v>1414</v>
       </c>
       <c r="O44" s="4" t="n">
         <v>0</v>
@@ -2876,10 +2876,10 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>43983</v>
+        <v>43770</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -2887,10 +2887,10 @@
         </is>
       </c>
       <c r="I45" s="3" t="n">
-        <v>46174</v>
+        <v>45962</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>46539</v>
+        <v>46327</v>
       </c>
       <c r="K45" s="4" t="n">
         <v>1240</v>
@@ -2899,10 +2899,10 @@
         <v>110</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>557</v>
+        <v>669</v>
       </c>
       <c r="N45" s="4" t="n">
-        <v>683</v>
+        <v>571</v>
       </c>
       <c r="O45" s="4" t="n">
         <v>0</v>
@@ -2983,10 +2983,10 @@
       </c>
       <c r="L48" s="6" t="inlineStr"/>
       <c r="M48" s="6" t="n">
-        <v>19798</v>
+        <v>19221</v>
       </c>
       <c r="N48" s="6" t="n">
-        <v>26379</v>
+        <v>26956</v>
       </c>
       <c r="O48" s="6" t="n">
         <v>0</v>

</xml_diff>